<commit_message>
Full 4 objectives model - Missing broadcasting Time Zone difference
</commit_message>
<xml_diff>
--- a/data_fifa.xlsx
+++ b/data_fifa.xlsx
@@ -253,27 +253,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau4" displayName="Tableau4" ref="A1:K17" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:K17"/>
-  <tableColumns count="11">
-    <tableColumn id="1" name="city"/>
-    <tableColumn id="2" name="stadium"/>
-    <tableColumn id="3" name="country"/>
-    <tableColumn id="4" name="let"/>
-    <tableColumn id="5" name="long"/>
-    <tableColumn id="6" name="alt_m"/>
-    <tableColumn id="7" name="capacity"/>
-    <tableColumn id="8" name="temp_C_june"/>
-    <tableColumn id="9" name="humidity_%_june"/>
-    <tableColumn id="10" name="time_zone"/>
-    <tableColumn id="11" name="UTC_Offset"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tableau1" displayName="Tableau1" ref="A1:K73" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau1" displayName="Tableau1" ref="A1:K73" headerRowCount="1" totalsRowShown="0">
   <sortState ref="A2:K73">
     <sortCondition ref="G1:G73"/>
   </sortState>
@@ -294,34 +274,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Tableau3" displayName="Tableau3" ref="A1:N49" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:N49"/>
-  <sortState ref="A2:I49">
-    <sortCondition ref="A1:A49"/>
-  </sortState>
-  <tableColumns count="14">
-    <tableColumn id="1" name="team"/>
-    <tableColumn id="2" name="group"/>
-    <tableColumn id="3" name="rank_fifa"/>
-    <tableColumn id="4" name="points_fifa"/>
-    <tableColumn id="5" name="federation"/>
-    <tableColumn id="6" name="capital_lat"/>
-    <tableColumn id="7" name="capital_long"/>
-    <tableColumn id="8" name="UTC_capital"/>
-    <tableColumn id="9" name="continent"/>
-    <tableColumn id="10" name="city_camp"/>
-    <tableColumn id="11" name="country_camp"/>
-    <tableColumn id="12" name="camp_name"/>
-    <tableColumn id="13" name="camp_lat"/>
-    <tableColumn id="14" name="camp_long"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Tableau2" displayName="Tableau2" ref="A1:F49" headerRowCount="1" totalsRowShown="0">
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Tableau2" displayName="Tableau2" ref="A1:F49" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A1:F49"/>
   <sortState ref="A2:F49">
     <sortCondition ref="A1:A49"/>
@@ -659,20 +613,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <cols>
-    <col width="43.5" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="31.83203125" customWidth="1" min="2" max="2"/>
-    <col width="15.6640625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="11.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="32.33203125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="14.33203125" customWidth="1" min="8" max="8"/>
-    <col width="17.33203125" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="43.5" bestFit="1" customWidth="1" min="12" max="12"/>
-  </cols>
+  <dimension ref="A1:L17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -730,6 +672,11 @@
           <t>UTC_Offset</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>elevation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -773,6 +720,9 @@
       <c r="K2" t="n">
         <v>-6</v>
       </c>
+      <c r="L2" t="n">
+        <v>2251</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -816,6 +766,9 @@
       <c r="K3" t="n">
         <v>-6</v>
       </c>
+      <c r="L3" t="n">
+        <v>1665</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -859,6 +812,9 @@
       <c r="K4" t="n">
         <v>-6</v>
       </c>
+      <c r="L4" t="n">
+        <v>494</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -902,6 +858,9 @@
       <c r="K5" t="n">
         <v>-5</v>
       </c>
+      <c r="L5" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -945,6 +904,9 @@
       <c r="K6" t="n">
         <v>-5</v>
       </c>
+      <c r="L6" t="n">
+        <v>193</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -988,6 +950,9 @@
       <c r="K7" t="n">
         <v>-5</v>
       </c>
+      <c r="L7" t="n">
+        <v>259</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1031,6 +996,9 @@
       <c r="K8" t="n">
         <v>-4</v>
       </c>
+      <c r="L8" t="n">
+        <v>316</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1074,6 +1042,9 @@
       <c r="K9" t="n">
         <v>-4</v>
       </c>
+      <c r="L9" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1117,6 +1088,9 @@
       <c r="K10" t="n">
         <v>-7</v>
       </c>
+      <c r="L10" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1160,6 +1134,9 @@
       <c r="K11" t="n">
         <v>-7</v>
       </c>
+      <c r="L11" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1203,6 +1180,9 @@
       <c r="K12" t="n">
         <v>-7</v>
       </c>
+      <c r="L12" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1246,6 +1226,9 @@
       <c r="K13" t="n">
         <v>-4</v>
       </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1289,6 +1272,9 @@
       <c r="K14" t="n">
         <v>-4</v>
       </c>
+      <c r="L14" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1332,6 +1318,9 @@
       <c r="K15" t="n">
         <v>-4</v>
       </c>
+      <c r="L15" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1375,6 +1364,9 @@
       <c r="K16" t="n">
         <v>-4</v>
       </c>
+      <c r="L16" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1418,60 +1410,12 @@
       <c r="K17" t="n">
         <v>-7</v>
       </c>
-    </row>
-    <row r="19" ht="19" customHeight="1">
-      <c r="A19" s="1" t="n"/>
-      <c r="L19" s="1" t="n"/>
-    </row>
-    <row r="20" ht="19" customHeight="1">
-      <c r="A20" s="1" t="n"/>
-      <c r="L20" s="1" t="n"/>
-    </row>
-    <row r="21" ht="19" customHeight="1">
-      <c r="A21" s="1" t="n"/>
-      <c r="L21" s="1" t="n"/>
-    </row>
-    <row r="22" ht="19" customHeight="1">
-      <c r="A22" s="1" t="n"/>
-      <c r="L22" s="1" t="n"/>
-    </row>
-    <row r="23" ht="19" customHeight="1">
-      <c r="A23" s="1" t="n"/>
-      <c r="L23" s="1" t="n"/>
-    </row>
-    <row r="24" ht="19" customHeight="1">
-      <c r="A24" s="1" t="n"/>
-      <c r="L24" s="1" t="n"/>
-    </row>
-    <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="1" t="n"/>
-      <c r="L25" s="1" t="n"/>
-    </row>
-    <row r="26" ht="19" customHeight="1">
-      <c r="A26" s="1" t="n"/>
-      <c r="L26" s="1" t="n"/>
-    </row>
-    <row r="27" ht="19" customHeight="1">
-      <c r="A27" s="1" t="n"/>
-      <c r="L27" s="1" t="n"/>
-    </row>
-    <row r="28" ht="19" customHeight="1">
-      <c r="A28" s="1" t="n"/>
-      <c r="L28" s="1" t="n"/>
-    </row>
-    <row r="29" ht="19" customHeight="1">
-      <c r="A29" s="1" t="n"/>
-      <c r="L29" s="1" t="n"/>
-    </row>
-    <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="1" t="n"/>
-      <c r="L30" s="1" t="n"/>
+      <c r="L17" t="n">
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -8622,16 +8566,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <cols>
-    <col width="12.33203125" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12.1640625" customWidth="1" min="6" max="6"/>
-    <col width="13.5" customWidth="1" min="7" max="7"/>
-    <col width="13.33203125" customWidth="1" min="8" max="8"/>
-    <col width="11.33203125" customWidth="1" min="9" max="9"/>
-  </cols>
+  <dimension ref="A1:P49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -8704,6 +8640,16 @@
           <t>camp_long</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>camp_elevation</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>camp_avg_temperature</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8756,15 +8702,17 @@
           <t>University of Kansas</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>38.9543</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>-95.2558</t>
-        </is>
+      <c r="M2" t="n">
+        <v>38.9543</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-95.25579999999999</v>
+      </c>
+      <c r="O2" t="n">
+        <v>287</v>
+      </c>
+      <c r="P2" t="n">
+        <v>27.72978070175438</v>
       </c>
     </row>
     <row r="3">
@@ -8818,15 +8766,17 @@
           <t>Sporting KC Training Centre</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>38.9714</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>-94.8113</t>
-        </is>
+      <c r="M3" t="n">
+        <v>38.9714</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-94.8113</v>
+      </c>
+      <c r="O3" t="n">
+        <v>281</v>
+      </c>
+      <c r="P3" t="n">
+        <v>27.33859649122807</v>
       </c>
     </row>
     <row r="4">
@@ -8880,15 +8830,17 @@
           <t>Oakland Roots/Soul Training Facility</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>37.7505</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>-122.1965</t>
-        </is>
+      <c r="M4" t="n">
+        <v>37.7505</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-122.1965</v>
+      </c>
+      <c r="O4" t="n">
+        <v>9</v>
+      </c>
+      <c r="P4" t="n">
+        <v>15.42530701754386</v>
       </c>
     </row>
     <row r="5">
@@ -8942,15 +8894,17 @@
           <t>UC Santa Barbara - Harder Stadium</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>34.4128</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>-119.8455</t>
-        </is>
+      <c r="M5" t="n">
+        <v>34.4128</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-119.8455</v>
+      </c>
+      <c r="O5" t="n">
+        <v>22</v>
+      </c>
+      <c r="P5" t="n">
+        <v>21.64872807017544</v>
       </c>
     </row>
     <row r="6">
@@ -9004,15 +8958,17 @@
           <t>Seattle Sounders FC Performance Centre and Clubhouse</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>47.4995</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>-122.2270</t>
-        </is>
+      <c r="M6" t="n">
+        <v>47.4995</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-122.227</v>
+      </c>
+      <c r="O6" t="n">
+        <v>42</v>
+      </c>
+      <c r="P6" t="n">
+        <v>14.96535087719298</v>
       </c>
     </row>
     <row r="7">
@@ -9066,15 +9022,17 @@
           <t>RSL Stadium</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>40.5829</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>-111.8932</t>
-        </is>
+      <c r="M7" t="n">
+        <v>40.5829</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-111.8932</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1350</v>
+      </c>
+      <c r="P7" t="n">
+        <v>20.81877192982456</v>
       </c>
     </row>
     <row r="8">
@@ -9128,15 +9086,17 @@
           <t>Columbia Park Training Facility</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>40.7920</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>-74.0539</t>
-        </is>
+      <c r="M8" t="n">
+        <v>40.792</v>
+      </c>
+      <c r="N8" t="n">
+        <v>-74.0539</v>
+      </c>
+      <c r="O8" t="n">
+        <v>4</v>
+      </c>
+      <c r="P8" t="n">
+        <v>22.61214912280701</v>
       </c>
     </row>
     <row r="9">
@@ -9190,15 +9150,17 @@
           <t>National Soccer Development Centre</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>49.2444</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>-123.2510</t>
-        </is>
+      <c r="M9" t="n">
+        <v>49.2444</v>
+      </c>
+      <c r="N9" t="n">
+        <v>-123.251</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>15.60359649122807</v>
       </c>
     </row>
     <row r="10">
@@ -9252,15 +9214,17 @@
           <t>Waters Sportsplex</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>28.0390</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>-82.5200</t>
-        </is>
+      <c r="M10" t="n">
+        <v>28.039</v>
+      </c>
+      <c r="N10" t="n">
+        <v>-82.52</v>
+      </c>
+      <c r="O10" t="n">
+        <v>13</v>
+      </c>
+      <c r="P10" t="n">
+        <v>31.20070175438597</v>
       </c>
     </row>
     <row r="11">
@@ -9314,15 +9278,17 @@
           <t>Academia Atlas FC</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>20.6258</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>-103.3450</t>
-        </is>
+      <c r="M11" t="n">
+        <v>20.6258</v>
+      </c>
+      <c r="N11" t="n">
+        <v>-103.345</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1566</v>
+      </c>
+      <c r="P11" t="n">
+        <v>23.53057017543859</v>
       </c>
     </row>
     <row r="12">
@@ -9376,15 +9342,17 @@
           <t>Episcopal High School</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>38.8080</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>-77.1030</t>
-        </is>
+      <c r="M12" t="n">
+        <v>38.808</v>
+      </c>
+      <c r="N12" t="n">
+        <v>-77.10299999999999</v>
+      </c>
+      <c r="O12" t="n">
+        <v>15</v>
+      </c>
+      <c r="P12" t="n">
+        <v>25.29872807017544</v>
       </c>
     </row>
     <row r="13">
@@ -9438,15 +9406,17 @@
           <t>Florida Atlantic University</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>26.3705</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>-80.1020</t>
-        </is>
+      <c r="M13" t="n">
+        <v>26.3705</v>
+      </c>
+      <c r="N13" t="n">
+        <v>-80.102</v>
+      </c>
+      <c r="O13" t="n">
+        <v>8</v>
+      </c>
+      <c r="P13" t="n">
+        <v>31.06456140350877</v>
       </c>
     </row>
     <row r="14">
@@ -9500,15 +9470,17 @@
           <t>Mansfield Multipurpose Stadium</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>32.5550</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>-97.1440</t>
-        </is>
+      <c r="M14" t="n">
+        <v>32.555</v>
+      </c>
+      <c r="N14" t="n">
+        <v>-97.14400000000001</v>
+      </c>
+      <c r="O14" t="n">
+        <v>200</v>
+      </c>
+      <c r="P14" t="n">
+        <v>31.53666666666667</v>
       </c>
     </row>
     <row r="15">
@@ -9562,15 +9534,17 @@
           <t>Houston Training Centre</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>29.6280</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>-95.3820</t>
-        </is>
+      <c r="M15" t="n">
+        <v>29.628</v>
+      </c>
+      <c r="N15" t="n">
+        <v>-95.38200000000001</v>
+      </c>
+      <c r="O15" t="n">
+        <v>13</v>
+      </c>
+      <c r="P15" t="n">
+        <v>32.90864035087719</v>
       </c>
     </row>
     <row r="16">
@@ -9624,15 +9598,17 @@
           <t>Columbus Crew Performance Centre</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>39.8570</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>-82.9670</t>
-        </is>
+      <c r="M16" t="n">
+        <v>39.857</v>
+      </c>
+      <c r="N16" t="n">
+        <v>-82.967</v>
+      </c>
+      <c r="O16" t="n">
+        <v>225</v>
+      </c>
+      <c r="P16" t="n">
+        <v>23.94311403508772</v>
       </c>
     </row>
     <row r="17">
@@ -9686,15 +9662,17 @@
           <t>Gonzaga University</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>47.6680</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>-117.3985</t>
-        </is>
+      <c r="M17" t="n">
+        <v>47.668</v>
+      </c>
+      <c r="N17" t="n">
+        <v>-117.3985</v>
+      </c>
+      <c r="O17" t="n">
+        <v>584</v>
+      </c>
+      <c r="P17" t="n">
+        <v>16.49184210526316</v>
       </c>
     </row>
     <row r="18">
@@ -9748,15 +9726,17 @@
           <t>Swope Soccer Village</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>39.0247</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>-94.5394</t>
-        </is>
+      <c r="M18" t="n">
+        <v>39.0247</v>
+      </c>
+      <c r="N18" t="n">
+        <v>-94.5394</v>
+      </c>
+      <c r="O18" t="n">
+        <v>281</v>
+      </c>
+      <c r="P18" t="n">
+        <v>27.67254385964912</v>
       </c>
     </row>
     <row r="19">
@@ -9810,15 +9790,17 @@
           <t>Bentley University</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>42.3905</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>-71.2210</t>
-        </is>
+      <c r="M19" t="n">
+        <v>42.3905</v>
+      </c>
+      <c r="N19" t="n">
+        <v>-71.221</v>
+      </c>
+      <c r="O19" t="n">
+        <v>64</v>
+      </c>
+      <c r="P19" t="n">
+        <v>20.81912280701754</v>
       </c>
     </row>
     <row r="20">
@@ -9872,15 +9854,17 @@
           <t>Wake Forest University</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>36.1352</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>-80.2789</t>
-        </is>
+      <c r="M20" t="n">
+        <v>36.1352</v>
+      </c>
+      <c r="N20" t="n">
+        <v>-80.27889999999999</v>
+      </c>
+      <c r="O20" t="n">
+        <v>292</v>
+      </c>
+      <c r="P20" t="n">
+        <v>26.01802631578947</v>
       </c>
     </row>
     <row r="21">
@@ -9934,15 +9918,17 @@
           <t>Bryant University</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>41.9173</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>-71.5350</t>
-        </is>
+      <c r="M21" t="n">
+        <v>41.9173</v>
+      </c>
+      <c r="N21" t="n">
+        <v>-71.535</v>
+      </c>
+      <c r="O21" t="n">
+        <v>126</v>
+      </c>
+      <c r="P21" t="n">
+        <v>20.56043859649123</v>
       </c>
     </row>
     <row r="22">
@@ -9996,15 +9982,17 @@
           <t>Stockton University</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>39.5010</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>-74.5350</t>
-        </is>
+      <c r="M22" t="n">
+        <v>39.501</v>
+      </c>
+      <c r="N22" t="n">
+        <v>-74.535</v>
+      </c>
+      <c r="O22" t="n">
+        <v>25</v>
+      </c>
+      <c r="P22" t="n">
+        <v>23.67236842105263</v>
       </c>
     </row>
     <row r="23">
@@ -10058,15 +10046,17 @@
           <t>Centro Xoloitzcuintle</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>32.4793</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>-116.8789</t>
-        </is>
+      <c r="M23" t="n">
+        <v>32.4793</v>
+      </c>
+      <c r="N23" t="n">
+        <v>-116.8789</v>
+      </c>
+      <c r="O23" t="n">
+        <v>164</v>
+      </c>
+      <c r="P23" t="n">
+        <v>20.03618421052632</v>
       </c>
     </row>
     <row r="24">
@@ -10120,15 +10110,17 @@
           <t>The Greenbrier Sports Performance Centre</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>37.7810</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>-80.2970</t>
-        </is>
+      <c r="M24" t="n">
+        <v>37.781</v>
+      </c>
+      <c r="N24" t="n">
+        <v>-80.297</v>
+      </c>
+      <c r="O24" t="n">
+        <v>663</v>
+      </c>
+      <c r="P24" t="n">
+        <v>20.83815789473684</v>
       </c>
     </row>
     <row r="25">
@@ -10182,15 +10174,17 @@
           <t>Philadelphia Union</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>39.8322</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>-75.3784</t>
-        </is>
+      <c r="M25" t="n">
+        <v>39.8322</v>
+      </c>
+      <c r="N25" t="n">
+        <v>-75.3784</v>
+      </c>
+      <c r="O25" t="n">
+        <v>10</v>
+      </c>
+      <c r="P25" t="n">
+        <v>24.00486842105263</v>
       </c>
     </row>
     <row r="26">
@@ -10244,15 +10238,17 @@
           <t>Nashville SC</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>36.1300</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>-86.7660</t>
-        </is>
+      <c r="M26" t="n">
+        <v>36.13</v>
+      </c>
+      <c r="N26" t="n">
+        <v>-86.76600000000001</v>
+      </c>
+      <c r="O26" t="n">
+        <v>155</v>
+      </c>
+      <c r="P26" t="n">
+        <v>27.67162280701755</v>
       </c>
     </row>
     <row r="27">
@@ -10306,15 +10302,17 @@
           <t>University of Portland</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>45.5720</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>-122.7265</t>
-        </is>
+      <c r="M27" t="n">
+        <v>45.572</v>
+      </c>
+      <c r="N27" t="n">
+        <v>-122.7265</v>
+      </c>
+      <c r="O27" t="n">
+        <v>54</v>
+      </c>
+      <c r="P27" t="n">
+        <v>16.70714912280702</v>
       </c>
     </row>
     <row r="28">
@@ -10368,15 +10366,17 @@
           <t>Chivas Verde Valle</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>20.6830</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>-103.4300</t>
-        </is>
+      <c r="M28" t="n">
+        <v>20.683</v>
+      </c>
+      <c r="N28" t="n">
+        <v>-103.43</v>
+      </c>
+      <c r="O28" t="n">
+        <v>1644</v>
+      </c>
+      <c r="P28" t="n">
+        <v>22.49166666666667</v>
       </c>
     </row>
     <row r="29">
@@ -10430,15 +10430,17 @@
           <t>Centro de Alto Rendimiento (CAR)</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>19.4070</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>-99.0980</t>
-        </is>
+      <c r="M29" t="n">
+        <v>19.407</v>
+      </c>
+      <c r="N29" t="n">
+        <v>-99.098</v>
+      </c>
+      <c r="O29" t="n">
+        <v>2231</v>
+      </c>
+      <c r="P29" t="n">
+        <v>17.85236842105263</v>
       </c>
     </row>
     <row r="30">
@@ -10492,15 +10494,17 @@
           <t>The Pingry School</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>40.6680</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>-74.5810</t>
-        </is>
+      <c r="M30" t="n">
+        <v>40.668</v>
+      </c>
+      <c r="N30" t="n">
+        <v>-74.581</v>
+      </c>
+      <c r="O30" t="n">
+        <v>90</v>
+      </c>
+      <c r="P30" t="n">
+        <v>22.53675438596492</v>
       </c>
     </row>
     <row r="31">
@@ -10554,15 +10558,17 @@
           <t>KC Current Training Facility</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>39.1490</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>-94.6090</t>
-        </is>
+      <c r="M31" t="n">
+        <v>39.149</v>
+      </c>
+      <c r="N31" t="n">
+        <v>-94.60899999999999</v>
+      </c>
+      <c r="O31" t="n">
+        <v>227</v>
+      </c>
+      <c r="P31" t="n">
+        <v>27.63188596491228</v>
       </c>
     </row>
     <row r="32">
@@ -10616,15 +10622,17 @@
           <t>University of San Diego - Torero Stadium</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>32.7700</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>-117.1875</t>
-        </is>
+      <c r="M32" t="n">
+        <v>32.77</v>
+      </c>
+      <c r="N32" t="n">
+        <v>-117.1875</v>
+      </c>
+      <c r="O32" t="n">
+        <v>66</v>
+      </c>
+      <c r="P32" t="n">
+        <v>19.3734649122807</v>
       </c>
     </row>
     <row r="33">
@@ -10678,15 +10686,17 @@
           <t>UNC Greensboro</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>36.0688</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>-79.8080</t>
-        </is>
+      <c r="M33" t="n">
+        <v>36.0688</v>
+      </c>
+      <c r="N33" t="n">
+        <v>-79.80800000000001</v>
+      </c>
+      <c r="O33" t="n">
+        <v>249</v>
+      </c>
+      <c r="P33" t="n">
+        <v>26.04934210526316</v>
       </c>
     </row>
     <row r="34">
@@ -10740,15 +10750,17 @@
           <t>Nottawasaga Training Site</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>44.1430</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>-79.8660</t>
-        </is>
+      <c r="M34" t="n">
+        <v>44.143</v>
+      </c>
+      <c r="N34" t="n">
+        <v>-79.866</v>
+      </c>
+      <c r="O34" t="n">
+        <v>221</v>
+      </c>
+      <c r="P34" t="n">
+        <v>19.19587719298245</v>
       </c>
     </row>
     <row r="35">
@@ -10802,15 +10814,17 @@
           <t>Spartan Soccer Complex</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>37.3460</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>-121.9285</t>
-        </is>
+      <c r="M35" t="n">
+        <v>37.346</v>
+      </c>
+      <c r="N35" t="n">
+        <v>-121.9285</v>
+      </c>
+      <c r="O35" t="n">
+        <v>22</v>
+      </c>
+      <c r="P35" t="n">
+        <v>18.70649122807018</v>
       </c>
     </row>
     <row r="36">
@@ -10864,15 +10878,17 @@
           <t>Gardens North County District Park</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>26.8915</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>-80.1350</t>
-        </is>
+      <c r="M36" t="n">
+        <v>26.8915</v>
+      </c>
+      <c r="N36" t="n">
+        <v>-80.13500000000001</v>
+      </c>
+      <c r="O36" t="n">
+        <v>5</v>
+      </c>
+      <c r="P36" t="n">
+        <v>30.87605263157894</v>
       </c>
     </row>
     <row r="37">
@@ -10926,15 +10942,17 @@
           <t>Westmont College</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>34.4427</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>-119.6610</t>
-        </is>
+      <c r="M37" t="n">
+        <v>34.4427</v>
+      </c>
+      <c r="N37" t="n">
+        <v>-119.661</v>
+      </c>
+      <c r="O37" t="n">
+        <v>157</v>
+      </c>
+      <c r="P37" t="n">
+        <v>21.21425438596491</v>
       </c>
     </row>
     <row r="38">
@@ -10988,15 +11006,17 @@
           <t>Austin FC Stadium</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>30.3881</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>-97.7196</t>
-        </is>
+      <c r="M38" t="n">
+        <v>30.3881</v>
+      </c>
+      <c r="N38" t="n">
+        <v>-97.7196</v>
+      </c>
+      <c r="O38" t="n">
+        <v>233</v>
+      </c>
+      <c r="P38" t="n">
+        <v>31.62894736842105</v>
       </c>
     </row>
     <row r="39">
@@ -11050,15 +11070,17 @@
           <t>Charlotte FC</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>35.2253</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>-80.8530</t>
-        </is>
+      <c r="M39" t="n">
+        <v>35.2253</v>
+      </c>
+      <c r="N39" t="n">
+        <v>-80.85299999999999</v>
+      </c>
+      <c r="O39" t="n">
+        <v>220</v>
+      </c>
+      <c r="P39" t="n">
+        <v>26.99122807017544</v>
       </c>
     </row>
     <row r="40">
@@ -11112,15 +11134,17 @@
           <t>Rutgers University</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>40.5240</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>-74.4350</t>
-        </is>
+      <c r="M40" t="n">
+        <v>40.524</v>
+      </c>
+      <c r="N40" t="n">
+        <v>-74.435</v>
+      </c>
+      <c r="O40" t="n">
+        <v>38</v>
+      </c>
+      <c r="P40" t="n">
+        <v>23.13083333333334</v>
       </c>
     </row>
     <row r="41">
@@ -11174,15 +11198,17 @@
           <t>CF Pachuca - Universidad Del Futbol</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>20.0901</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>-98.7536</t>
-        </is>
+      <c r="M41" t="n">
+        <v>20.0901</v>
+      </c>
+      <c r="N41" t="n">
+        <v>-98.75360000000001</v>
+      </c>
+      <c r="O41" t="n">
+        <v>2365</v>
+      </c>
+      <c r="P41" t="n">
+        <v>15.16754385964912</v>
       </c>
     </row>
     <row r="42">
@@ -11236,15 +11262,17 @@
           <t>Baylor School</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>35.0822</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>-85.2980</t>
-        </is>
+      <c r="M42" t="n">
+        <v>35.0822</v>
+      </c>
+      <c r="N42" t="n">
+        <v>-85.298</v>
+      </c>
+      <c r="O42" t="n">
+        <v>270</v>
+      </c>
+      <c r="P42" t="n">
+        <v>26.71934210526316</v>
       </c>
     </row>
     <row r="43">
@@ -11298,15 +11326,17 @@
           <t>FC Dallas Stadium</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>33.1546</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>-96.8350</t>
-        </is>
+      <c r="M43" t="n">
+        <v>33.1546</v>
+      </c>
+      <c r="N43" t="n">
+        <v>-96.83499999999999</v>
+      </c>
+      <c r="O43" t="n">
+        <v>186</v>
+      </c>
+      <c r="P43" t="n">
+        <v>31.31171052631579</v>
       </c>
     </row>
     <row r="44">
@@ -11360,15 +11390,17 @@
           <t>SDJA</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>32.9481</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>-117.2340</t>
-        </is>
+      <c r="M44" t="n">
+        <v>32.9481</v>
+      </c>
+      <c r="N44" t="n">
+        <v>-117.234</v>
+      </c>
+      <c r="O44" t="n">
+        <v>66</v>
+      </c>
+      <c r="P44" t="n">
+        <v>19.70504385964912</v>
       </c>
     </row>
     <row r="45">
@@ -11422,15 +11454,17 @@
           <t>Rayados Training Centre</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>25.7220</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>-100.2470</t>
-        </is>
+      <c r="M45" t="n">
+        <v>25.722</v>
+      </c>
+      <c r="N45" t="n">
+        <v>-100.247</v>
+      </c>
+      <c r="O45" t="n">
+        <v>479</v>
+      </c>
+      <c r="P45" t="n">
+        <v>30.49228070175438</v>
       </c>
     </row>
     <row r="46">
@@ -11484,15 +11518,17 @@
           <t>Arizona Athletic Grounds</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>33.3550</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>-111.6830</t>
-        </is>
+      <c r="M46" t="n">
+        <v>33.355</v>
+      </c>
+      <c r="N46" t="n">
+        <v>-111.683</v>
+      </c>
+      <c r="O46" t="n">
+        <v>405</v>
+      </c>
+      <c r="P46" t="n">
+        <v>31.62574561403509</v>
       </c>
     </row>
     <row r="47">
@@ -11546,15 +11582,17 @@
           <t>Mayakoba Training Centre Cancun</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>20.7010</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>-87.0240</t>
-        </is>
+      <c r="M47" t="n">
+        <v>20.701</v>
+      </c>
+      <c r="N47" t="n">
+        <v>-87.024</v>
+      </c>
+      <c r="O47" t="n">
+        <v>14</v>
+      </c>
+      <c r="P47" t="n">
+        <v>31.97087719298246</v>
       </c>
     </row>
     <row r="48">
@@ -11608,15 +11646,17 @@
           <t>Great Park Sports Complex</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>33.6713</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>-117.7410</t>
-        </is>
+      <c r="M48" t="n">
+        <v>33.6713</v>
+      </c>
+      <c r="N48" t="n">
+        <v>-117.741</v>
+      </c>
+      <c r="O48" t="n">
+        <v>82</v>
+      </c>
+      <c r="P48" t="n">
+        <v>20.01982456140351</v>
       </c>
     </row>
     <row r="49">
@@ -11670,22 +11710,21 @@
           <t>Atlanta United Training Centre</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>33.9690</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>-84.5720</t>
-        </is>
+      <c r="M49" t="n">
+        <v>33.969</v>
+      </c>
+      <c r="N49" t="n">
+        <v>-84.572</v>
+      </c>
+      <c r="O49" t="n">
+        <v>338</v>
+      </c>
+      <c r="P49" t="n">
+        <v>26.88627192982456</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>